<commit_message>
Roaming xleda installation fix for Windows
</commit_message>
<xml_diff>
--- a/src/xleda/assets/xleda_template.xlsx
+++ b/src/xleda/assets/xleda_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB4A3E80-F33D-43AE-88FE-4CCEB7A1E027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{27416712-FCEE-487F-83CE-CBB073D1063A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
@@ -1078,7 +1078,7 @@
     </xf>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" textRotation="180"/>
@@ -1403,6 +1403,7 @@
     <xf numFmtId="0" fontId="36" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="3" fontId="32" fillId="2" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -4899,7 +4900,7 @@
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
     <col min="2" max="2" width="8.28515625" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
     <col min="5" max="6" width="27.28515625" customWidth="1"/>
     <col min="7" max="11" width="19.42578125" customWidth="1"/>
@@ -4909,10 +4910,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="5.0999999999999996" customHeight="1"/>
-    <row r="2" spans="1:28" ht="14.45" customHeight="1">
+    <row r="2" spans="1:28" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="70"/>
     </row>
-    <row r="3" spans="1:28" ht="10.35" customHeight="1">
+    <row r="3" spans="1:28" ht="5.0999999999999996" customHeight="1">
       <c r="A3" s="70"/>
     </row>
     <row r="4" spans="1:28" ht="30" customHeight="1">
@@ -4925,7 +4926,7 @@
       <c r="D4" s="73"/>
       <c r="AB4" s="4"/>
     </row>
-    <row r="5" spans="1:28" ht="20.100000000000001" customHeight="1">
+    <row r="5" spans="1:28" ht="10.35" customHeight="1">
       <c r="C5" s="53"/>
       <c r="AB5" s="4"/>
     </row>
@@ -4959,10 +4960,10 @@
       <c r="K8" s="43"/>
     </row>
     <row r="9" spans="1:28" ht="30" hidden="1" customHeight="1">
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="D9" s="116"/>
+      <c r="D9" s="117"/>
       <c r="E9" s="43"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -4988,10 +4989,10 @@
     </row>
     <row r="12" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="B12" s="1"/>
-      <c r="C12" s="116" t="s">
+      <c r="C12" s="117" t="s">
         <v>95</v>
       </c>
-      <c r="D12" s="116"/>
+      <c r="D12" s="117"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
       <c r="K12" s="43"/>
@@ -5045,10 +5046,10 @@
       <c r="L19" s="38"/>
     </row>
     <row r="20" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C20" s="116" t="s">
+      <c r="C20" s="117" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="116"/>
+      <c r="D20" s="117"/>
       <c r="E20" s="78"/>
       <c r="L20" s="38"/>
     </row>
@@ -5176,10 +5177,10 @@
       <c r="Y38" s="38"/>
     </row>
     <row r="39" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C39" s="116" t="s">
+      <c r="C39" s="117" t="s">
         <v>53</v>
       </c>
-      <c r="D39" s="116"/>
+      <c r="D39" s="117"/>
       <c r="F39" s="43"/>
       <c r="G39" s="43"/>
       <c r="H39" s="43"/>
@@ -5684,7 +5685,7 @@
   <sheetPr codeName="Sheet2">
     <tabColor rgb="FF131313"/>
   </sheetPr>
-  <dimension ref="B1:H83"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr defaultColWidth="15.7109375" defaultRowHeight="15" customHeight="1" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -5694,7 +5695,7 @@
     <col min="5" max="6" width="27.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="20.100000000000001" hidden="1" customHeight="1">
+    <row r="1" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1">
       <c r="B1" s="13"/>
       <c r="C1" s="14"/>
       <c r="D1" s="14" t="s">
@@ -5705,7 +5706,7 @@
       <c r="G1" s="14"/>
       <c r="H1" s="14"/>
     </row>
-    <row r="2" spans="2:8" ht="5.0999999999999996" customHeight="1">
+    <row r="2" spans="1:8" ht="5.0999999999999996" customHeight="1">
       <c r="C2" s="74"/>
       <c r="D2" s="74"/>
       <c r="E2" s="74"/>
@@ -5713,17 +5714,17 @@
       <c r="G2" s="74"/>
       <c r="H2" s="74"/>
     </row>
-    <row r="3" spans="2:8" ht="20.100000000000001" customHeight="1">
+    <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="B3" s="115" t="str">
         <f ca="1">HYPERLINK("#" &amp; CELL("address", _xlfn.XLOOKUP(Name,tbl_DfOverview[Dataframe],tbl_DfOverview[_],tbl_DfOverview[[#Headers],[_]])), "Overview →")</f>
         <v>Overview →</v>
       </c>
       <c r="C3" s="81"/>
     </row>
-    <row r="4" spans="2:8" ht="5.0999999999999996" customHeight="1">
+    <row r="4" spans="1:8" ht="5.0999999999999996" customHeight="1">
       <c r="B4" s="68"/>
     </row>
-    <row r="5" spans="2:8" ht="30" customHeight="1">
+    <row r="5" spans="1:8" ht="30" customHeight="1">
       <c r="B5" s="105" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -5732,8 +5733,9 @@
       </c>
       <c r="D5" s="22"/>
     </row>
-    <row r="6" spans="2:8" ht="10.35" customHeight="1"/>
-    <row r="7" spans="2:8">
+    <row r="6" spans="1:8" ht="10.35" customHeight="1"/>
+    <row r="7" spans="1:8">
+      <c r="A7" s="116"/>
       <c r="B7" s="82" t="s">
         <v>106</v>
       </c>
@@ -5741,46 +5743,59 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1"/>
-    <row r="9" spans="2:8" ht="50.1" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="A8" s="116"/>
+    </row>
+    <row r="9" spans="1:8" ht="50.1" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A9" s="116"/>
       <c r="D9" s="71" t="s">
         <v>51</v>
       </c>
       <c r="E9" s="72"/>
     </row>
-    <row r="10" spans="2:8" hidden="1" outlineLevel="1"/>
-    <row r="11" spans="2:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="10" spans="1:8" hidden="1" outlineLevel="1">
+      <c r="A10" s="116"/>
+    </row>
+    <row r="11" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A11" s="116"/>
       <c r="C11" s="21" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="32"/>
     </row>
-    <row r="12" spans="2:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="12" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A12" s="116"/>
       <c r="C12" s="3" t="s">
         <v>48</v>
       </c>
       <c r="D12" s="24"/>
     </row>
-    <row r="13" spans="2:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="13" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A13" s="116"/>
       <c r="C13" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="24"/>
     </row>
-    <row r="14" spans="2:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="14" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A14" s="116"/>
       <c r="C14" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D14" s="30"/>
     </row>
-    <row r="15" spans="2:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="15" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A15" s="116"/>
       <c r="C15" s="3" t="s">
         <v>50</v>
       </c>
       <c r="D15" s="31"/>
     </row>
-    <row r="16" spans="2:8" ht="10.35" hidden="1" customHeight="1" outlineLevel="1"/>
-    <row r="17" spans="2:6" ht="35.1" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="16" spans="1:8" ht="10.35" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A16" s="116"/>
+    </row>
+    <row r="17" spans="1:6" ht="35.1" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A17" s="116"/>
       <c r="C17" s="21" t="s">
         <v>2</v>
       </c>
@@ -5794,8 +5809,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="2:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="1"/>
-    <row r="19" spans="2:6" ht="35.1" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="18" spans="1:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A18" s="116"/>
+    </row>
+    <row r="19" spans="1:6" ht="35.1" hidden="1" customHeight="1" outlineLevel="1">
       <c r="C19" s="21" t="s">
         <v>3</v>
       </c>
@@ -5809,8 +5826,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="2:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="1"/>
-    <row r="21" spans="2:6" s="23" customFormat="1" ht="30" customHeight="1" collapsed="1">
+    <row r="20" spans="1:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="1"/>
+    <row r="21" spans="1:6" s="23" customFormat="1" ht="30" customHeight="1" collapsed="1">
       <c r="B21" s="58"/>
       <c r="C21" s="58" t="s">
         <v>4</v>
@@ -5819,8 +5836,9 @@
       <c r="E21" s="59"/>
       <c r="F21" s="59"/>
     </row>
-    <row r="22" spans="2:6" ht="10.35" customHeight="1"/>
-    <row r="23" spans="2:6" outlineLevel="1">
+    <row r="22" spans="1:6" ht="10.35" customHeight="1"/>
+    <row r="23" spans="1:6" outlineLevel="1">
+      <c r="A23" s="116"/>
       <c r="B23" s="82" t="s">
         <v>106</v>
       </c>
@@ -5828,8 +5846,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="2:6" ht="20.100000000000001" customHeight="1" outlineLevel="1"/>
-    <row r="25" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="24" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
+      <c r="A24" s="116"/>
+    </row>
+    <row r="25" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A25" s="116"/>
       <c r="C25" s="19" t="s">
         <v>8</v>
       </c>
@@ -5837,7 +5858,8 @@
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="26" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A26" s="116"/>
       <c r="C26" s="3" t="s">
         <v>9</v>
       </c>
@@ -5845,7 +5867,8 @@
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
     </row>
-    <row r="27" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="27" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A27" s="116"/>
       <c r="C27" s="18" t="s">
         <v>10</v>
       </c>
@@ -5853,7 +5876,8 @@
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
     </row>
-    <row r="28" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="28" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A28" s="116"/>
       <c r="C28" s="18" t="s">
         <v>11</v>
       </c>
@@ -5861,7 +5885,8 @@
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
     </row>
-    <row r="29" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="29" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A29" s="116"/>
       <c r="C29" s="18" t="s">
         <v>12</v>
       </c>
@@ -5869,7 +5894,8 @@
       <c r="E29" s="11"/>
       <c r="F29" s="11"/>
     </row>
-    <row r="30" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="30" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A30" s="116"/>
       <c r="C30" s="18" t="s">
         <v>13</v>
       </c>
@@ -5877,7 +5903,8 @@
       <c r="E30" s="11"/>
       <c r="F30" s="11"/>
     </row>
-    <row r="31" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="31" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A31" s="116"/>
       <c r="C31" s="19" t="s">
         <v>14</v>
       </c>
@@ -5885,7 +5912,8 @@
       <c r="E31" s="11"/>
       <c r="F31" s="11"/>
     </row>
-    <row r="32" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="32" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A32" s="116"/>
       <c r="C32" s="3" t="s">
         <v>15</v>
       </c>
@@ -5893,10 +5921,13 @@
       <c r="E32" s="11"/>
       <c r="F32" s="11"/>
     </row>
-    <row r="33" spans="2:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="34" spans="2:6" ht="125.1" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="35" spans="2:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="36" spans="2:6" outlineLevel="1" collapsed="1">
+    <row r="33" spans="1:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A33" s="116"/>
+    </row>
+    <row r="34" spans="1:6" ht="125.1" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="35" spans="1:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="36" spans="1:6" outlineLevel="1" collapsed="1">
+      <c r="A36" s="116"/>
       <c r="B36" s="82" t="s">
         <v>106</v>
       </c>
@@ -5904,8 +5935,11 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="2:6" ht="20.100000000000001" customHeight="1" outlineLevel="1"/>
-    <row r="38" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="37" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
+      <c r="A37" s="116"/>
+    </row>
+    <row r="38" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A38" s="116"/>
       <c r="C38" s="3" t="s">
         <v>17</v>
       </c>
@@ -5913,7 +5947,8 @@
       <c r="E38" s="12"/>
       <c r="F38" s="12"/>
     </row>
-    <row r="39" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="39" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A39" s="116"/>
       <c r="C39" s="18" t="s">
         <v>18</v>
       </c>
@@ -5921,7 +5956,8 @@
       <c r="E39" s="12"/>
       <c r="F39" s="12"/>
     </row>
-    <row r="40" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="40" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A40" s="116"/>
       <c r="C40" s="18" t="s">
         <v>19</v>
       </c>
@@ -5929,7 +5965,8 @@
       <c r="E40" s="12"/>
       <c r="F40" s="12"/>
     </row>
-    <row r="41" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="41" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A41" s="116"/>
       <c r="C41" s="3" t="s">
         <v>20</v>
       </c>
@@ -5937,7 +5974,8 @@
       <c r="E41" s="12"/>
       <c r="F41" s="12"/>
     </row>
-    <row r="42" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="42" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A42" s="116"/>
       <c r="C42" s="20" t="s">
         <v>21</v>
       </c>
@@ -5945,10 +5983,13 @@
       <c r="E42" s="12"/>
       <c r="F42" s="12"/>
     </row>
-    <row r="43" spans="2:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="44" spans="2:6" ht="150" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="45" spans="2:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="46" spans="2:6" outlineLevel="1" collapsed="1">
+    <row r="43" spans="1:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A43" s="116"/>
+    </row>
+    <row r="44" spans="1:6" ht="150" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="45" spans="1:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="46" spans="1:6" outlineLevel="1" collapsed="1">
+      <c r="A46" s="116"/>
       <c r="B46" s="82" t="s">
         <v>106</v>
       </c>
@@ -5956,8 +5997,11 @@
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="2:6" ht="20.100000000000001" customHeight="1" outlineLevel="1"/>
-    <row r="48" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="47" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
+      <c r="A47" s="116"/>
+    </row>
+    <row r="48" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A48" s="116"/>
       <c r="C48" s="3" t="s">
         <v>23</v>
       </c>
@@ -5965,7 +6009,8 @@
       <c r="E48" s="12"/>
       <c r="F48" s="12"/>
     </row>
-    <row r="49" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="49" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A49" s="116"/>
       <c r="C49" s="18">
         <v>0.05</v>
       </c>
@@ -5973,7 +6018,8 @@
       <c r="E49" s="12"/>
       <c r="F49" s="12"/>
     </row>
-    <row r="50" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="50" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A50" s="116"/>
       <c r="C50" s="19">
         <v>0.25</v>
       </c>
@@ -5981,7 +6027,8 @@
       <c r="E50" s="12"/>
       <c r="F50" s="12"/>
     </row>
-    <row r="51" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="51" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A51" s="116"/>
       <c r="C51" s="3">
         <v>0.5</v>
       </c>
@@ -5989,7 +6036,8 @@
       <c r="E51" s="12"/>
       <c r="F51" s="12"/>
     </row>
-    <row r="52" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="52" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A52" s="116"/>
       <c r="C52" s="18">
         <v>0.75</v>
       </c>
@@ -5997,7 +6045,8 @@
       <c r="E52" s="12"/>
       <c r="F52" s="12"/>
     </row>
-    <row r="53" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="53" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A53" s="116"/>
       <c r="C53" s="18">
         <v>0.95</v>
       </c>
@@ -6005,7 +6054,8 @@
       <c r="E53" s="12"/>
       <c r="F53" s="12"/>
     </row>
-    <row r="54" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="54" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A54" s="116"/>
       <c r="C54" s="3" t="s">
         <v>24</v>
       </c>
@@ -6013,7 +6063,8 @@
       <c r="E54" s="12"/>
       <c r="F54" s="12"/>
     </row>
-    <row r="55" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="55" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A55" s="116"/>
       <c r="C55" s="18" t="s">
         <v>25</v>
       </c>
@@ -6021,7 +6072,7 @@
       <c r="E55" s="12"/>
       <c r="F55" s="12"/>
     </row>
-    <row r="56" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="56" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
       <c r="C56" s="3" t="s">
         <v>26</v>
       </c>
@@ -6029,8 +6080,9 @@
       <c r="E56" s="12"/>
       <c r="F56" s="12"/>
     </row>
-    <row r="57" spans="2:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="58" spans="2:6" outlineLevel="1" collapsed="1">
+    <row r="57" spans="1:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="58" spans="1:6" outlineLevel="1" collapsed="1">
+      <c r="A58" s="116"/>
       <c r="B58" s="82" t="s">
         <v>106</v>
       </c>
@@ -6038,8 +6090,11 @@
         <v>27</v>
       </c>
     </row>
-    <row r="59" spans="2:6" ht="20.100000000000001" customHeight="1" outlineLevel="1"/>
-    <row r="60" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="59" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
+      <c r="A59" s="116"/>
+    </row>
+    <row r="60" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A60" s="116"/>
       <c r="C60" s="3" t="s">
         <v>28</v>
       </c>
@@ -6053,7 +6108,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="61" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A61" s="116"/>
       <c r="C61" s="18" t="s">
         <v>29</v>
       </c>
@@ -6067,7 +6123,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="62" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A62" s="116"/>
       <c r="C62" s="18" t="s">
         <v>30</v>
       </c>
@@ -6081,7 +6138,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="63" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A63" s="116"/>
       <c r="C63" s="18" t="s">
         <v>31</v>
       </c>
@@ -6095,7 +6153,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="64" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A64" s="116"/>
       <c r="C64" s="3" t="s">
         <v>32</v>
       </c>
@@ -6109,7 +6168,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="65" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A65" s="116"/>
       <c r="C65" s="18" t="s">
         <v>33</v>
       </c>
@@ -6123,7 +6183,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="66" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A66" s="116"/>
       <c r="C66" s="18" t="s">
         <v>34</v>
       </c>
@@ -6137,7 +6198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="67" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
       <c r="C67" s="3" t="s">
         <v>35</v>
       </c>
@@ -6151,8 +6212,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="2:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="69" spans="2:6" outlineLevel="1" collapsed="1">
+    <row r="68" spans="1:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="69" spans="1:6" outlineLevel="1" collapsed="1">
+      <c r="A69" s="116"/>
       <c r="B69" s="82" t="s">
         <v>106</v>
       </c>
@@ -6160,8 +6222,11 @@
         <v>36</v>
       </c>
     </row>
-    <row r="70" spans="2:6" ht="20.100000000000001" customHeight="1" outlineLevel="1"/>
-    <row r="71" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="70" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
+      <c r="A70" s="116"/>
+    </row>
+    <row r="71" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A71" s="116"/>
       <c r="C71" s="3" t="str">
         <f>IF(COUNTIF(FieldList1, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C60)," ","_") &amp;" = ")</f>
         <v/>
@@ -6171,7 +6236,8 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="72" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A72" s="116"/>
       <c r="C72" s="17" t="str">
         <f>IF(COUNTIF(FieldList2, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C61)," ","_")&amp;" = ")</f>
         <v/>
@@ -6181,7 +6247,8 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="73" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A73" s="116"/>
       <c r="C73" s="17" t="str">
         <f>IF(COUNTIF(FieldList3, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C62)," ","_")&amp;" = ")</f>
         <v/>
@@ -6191,7 +6258,8 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="74" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A74" s="116"/>
       <c r="C74" s="17" t="str">
         <f>IF(COUNTIF(FieldList4, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C63)," ","_")&amp;" = ")</f>
         <v/>
@@ -6201,7 +6269,8 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="75" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A75" s="116"/>
       <c r="C75" s="17" t="str">
         <f>IF(COUNTIF(FieldList5, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C64)," ","_")&amp;" = ")</f>
         <v/>
@@ -6211,7 +6280,8 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="76" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A76" s="116"/>
       <c r="C76" s="17" t="str">
         <f>IF(COUNTIF(FieldList6, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C65)," ","_")&amp;" = ")</f>
         <v/>
@@ -6221,7 +6291,8 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="77" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A77" s="116"/>
       <c r="C77" s="16" t="str">
         <f>IF(COUNTIF(FieldList7, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C66)," ","_")&amp;" = ")</f>
         <v/>
@@ -6231,7 +6302,8 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="78" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A78" s="116"/>
       <c r="C78" s="3" t="str">
         <f>IF(COUNTIF(FieldList8, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C67)," ","_")&amp;" = ")</f>
         <v/>
@@ -6241,7 +6313,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="2:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
+    <row r="79" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
       <c r="C79" s="15" t="str">
         <f>IF(COUNTIF(tbl_SourceData[Record List], "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(LightHeader)," ", "_") &amp;" = ")</f>
         <v/>
@@ -6251,7 +6323,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="2:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="1" collapsed="1"/>
+    <row r="80" spans="1:6" ht="10.35" hidden="1" customHeight="1" outlineLevel="1" collapsed="1"/>
     <row r="81" spans="3:6" ht="30" customHeight="1">
       <c r="C81" s="62" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Move PythonList to a lambda function
</commit_message>
<xml_diff>
--- a/src/xleda/assets/xleda_template.xlsx
+++ b/src/xleda/assets/xleda_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CB782DB-F52E-4735-BFE1-D6AB23CCF045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B025F63-C475-40D8-9EDC-409F212BDAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
@@ -54,6 +54,7 @@
     <definedName name="Name" localSheetId="0">SinglePlot!$C$4</definedName>
     <definedName name="Notes" localSheetId="2">'Field Analysis'!$D$19:$F$19</definedName>
     <definedName name="Percentiles" localSheetId="2">'Field Analysis'!$C$48:$C$57</definedName>
+    <definedName name="PythonList">_xlfn.LAMBDA(_xlpm.rng,     "[" &amp;      _xlfn.TEXTJOIN(", ", TRUE,          _xlfn.MAP(_xlpm.rng, _xlfn.LAMBDA(_xlpm.cell,             IF(OR(ISERROR(_xlpm.cell), ISBLANK(_xlpm.cell)), "''",             IF(ISLOGICAL(_xlpm.cell), IF(_xlpm.cell, "True", "False"),             IF(ISNUMBER(_xlpm.cell), _xlpm.cell,             "'" &amp; SUBSTITUTE(_xlpm.cell, "'", "\'") &amp; "'"             )))         ))     ) &amp;      "]" )</definedName>
     <definedName name="SerializedLists" localSheetId="2">'Field Analysis'!$D$71:$D$80</definedName>
     <definedName name="SinglePlot" localSheetId="0">SinglePlot!$C$10</definedName>
     <definedName name="Summary_Stats" localSheetId="2">'Field Analysis'!$C$38:$C$45</definedName>
@@ -6232,7 +6233,7 @@
         <v/>
       </c>
       <c r="D71" t="str" cm="1">
-        <f t="array" ref="D71">IF(COUNTIF(FieldList1, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList1&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D71">IF(COUNTIF(FieldList1, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList1&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6243,7 +6244,7 @@
         <v/>
       </c>
       <c r="D72" t="str" cm="1">
-        <f t="array" ref="D72">IF(COUNTIF(FieldList2, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList2&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D72">IF(COUNTIF(FieldList2, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList2&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6254,7 +6255,7 @@
         <v/>
       </c>
       <c r="D73" t="str" cm="1">
-        <f t="array" ref="D73">IF(COUNTIF(FieldList3, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList3&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D73">IF(COUNTIF(FieldList3, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList3&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6265,7 +6266,7 @@
         <v/>
       </c>
       <c r="D74" t="str" cm="1">
-        <f t="array" ref="D74">IF(COUNTIF(FieldList4, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList4&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D74">IF(COUNTIF(FieldList4, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList4&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6276,7 +6277,7 @@
         <v/>
       </c>
       <c r="D75" t="str" cm="1">
-        <f t="array" ref="D75">IF(COUNTIF(FieldList5, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList5&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D75">IF(COUNTIF(FieldList5, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList5&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6287,7 +6288,7 @@
         <v/>
       </c>
       <c r="D76" t="str" cm="1">
-        <f t="array" ref="D76">IF(COUNTIF(FieldList6, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList6&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D76">IF(COUNTIF(FieldList6, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList6&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6298,7 +6299,7 @@
         <v/>
       </c>
       <c r="D77" t="str" cm="1">
-        <f t="array" ref="D77">IF(COUNTIF(FieldList7, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList7&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D77">IF(COUNTIF(FieldList7, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList7&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6309,7 +6310,7 @@
         <v/>
       </c>
       <c r="D78" t="str" cm="1">
-        <f t="array" ref="D78">IF(COUNTIF(FieldList8, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList8&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D78">IF(COUNTIF(FieldList8, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList8&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6319,7 +6320,7 @@
         <v/>
       </c>
       <c r="D79" t="str" cm="1">
-        <f t="array" ref="D79">IF(COUNTIF(tbl_SourceData[Record List], "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(_xlfn.TAKE(tbl_SourceData[],,-1), tbl_SourceData[Record List] &lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D79">IF(COUNTIF(tbl_SourceData[Record List], "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(_xlfn.TAKE(tbl_SourceData[],,-1), tbl_SourceData[Record List] &lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Move PythonList to a lambda function Tiny readme updates
</commit_message>
<xml_diff>
--- a/src/xleda/assets/xleda_template.xlsx
+++ b/src/xleda/assets/xleda_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CB782DB-F52E-4735-BFE1-D6AB23CCF045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DEC2917-5243-4B12-BB72-D67C3A2954B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
@@ -54,6 +54,7 @@
     <definedName name="Name" localSheetId="0">SinglePlot!$C$4</definedName>
     <definedName name="Notes" localSheetId="2">'Field Analysis'!$D$19:$F$19</definedName>
     <definedName name="Percentiles" localSheetId="2">'Field Analysis'!$C$48:$C$57</definedName>
+    <definedName name="PythonList">_xlfn.LAMBDA(_xlpm.rng,     "[" &amp;      _xlfn.TEXTJOIN(", ", TRUE,          _xlfn.MAP(_xlpm.rng, _xlfn.LAMBDA(_xlpm.cell,             IF(OR(ISERROR(_xlpm.cell), ISBLANK(_xlpm.cell)), "''",             IF(ISLOGICAL(_xlpm.cell), IF(_xlpm.cell, "True", "False"),             IF(ISNUMBER(_xlpm.cell), _xlpm.cell,             "'" &amp; SUBSTITUTE(_xlpm.cell, "'", "\'") &amp; "'"             )))         ))     ) &amp;      "]" )</definedName>
     <definedName name="SerializedLists" localSheetId="2">'Field Analysis'!$D$71:$D$80</definedName>
     <definedName name="SinglePlot" localSheetId="0">SinglePlot!$C$10</definedName>
     <definedName name="Summary_Stats" localSheetId="2">'Field Analysis'!$C$38:$C$45</definedName>
@@ -6232,7 +6233,7 @@
         <v/>
       </c>
       <c r="D71" t="str" cm="1">
-        <f t="array" ref="D71">IF(COUNTIF(FieldList1, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList1&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D71">IF(COUNTIF(FieldList1, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList1&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6243,7 +6244,7 @@
         <v/>
       </c>
       <c r="D72" t="str" cm="1">
-        <f t="array" ref="D72">IF(COUNTIF(FieldList2, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList2&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D72">IF(COUNTIF(FieldList2, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList2&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6254,7 +6255,7 @@
         <v/>
       </c>
       <c r="D73" t="str" cm="1">
-        <f t="array" ref="D73">IF(COUNTIF(FieldList3, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList3&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D73">IF(COUNTIF(FieldList3, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList3&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6265,7 +6266,7 @@
         <v/>
       </c>
       <c r="D74" t="str" cm="1">
-        <f t="array" ref="D74">IF(COUNTIF(FieldList4, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList4&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D74">IF(COUNTIF(FieldList4, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList4&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6276,7 +6277,7 @@
         <v/>
       </c>
       <c r="D75" t="str" cm="1">
-        <f t="array" ref="D75">IF(COUNTIF(FieldList5, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList5&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D75">IF(COUNTIF(FieldList5, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList5&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6287,7 +6288,7 @@
         <v/>
       </c>
       <c r="D76" t="str" cm="1">
-        <f t="array" ref="D76">IF(COUNTIF(FieldList6, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList6&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D76">IF(COUNTIF(FieldList6, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList6&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6298,7 +6299,7 @@
         <v/>
       </c>
       <c r="D77" t="str" cm="1">
-        <f t="array" ref="D77">IF(COUNTIF(FieldList7, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList7&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D77">IF(COUNTIF(FieldList7, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList7&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6309,7 +6310,7 @@
         <v/>
       </c>
       <c r="D78" t="str" cm="1">
-        <f t="array" ref="D78">IF(COUNTIF(FieldList8, "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(FieldRange,FieldList8&lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D78">IF(COUNTIF(FieldList8, "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(FieldRange,FieldList8&lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>
@@ -6319,7 +6320,7 @@
         <v/>
       </c>
       <c r="D79" t="str" cm="1">
-        <f t="array" ref="D79">IF(COUNTIF(tbl_SourceData[Record List], "&lt;&gt;FALSE") = 0,"","['"&amp;_xlfn.TEXTJOIN("', '", TRUE, _xlfn._xlws.FILTER(_xlfn.TAKE(tbl_SourceData[],,-1), tbl_SourceData[Record List] &lt;&gt; FALSE, ""))&amp;"']")</f>
+        <f t="array" ref="D79">IF(COUNTIF(tbl_SourceData[Record List], "&lt;&gt;FALSE") = 0,"",PythonList(_xlfn._xlws.FILTER(_xlfn.TAKE(tbl_SourceData[],,-1), tbl_SourceData[Record List] &lt;&gt; FALSE, "")))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Typo correction on readme, link updates
</commit_message>
<xml_diff>
--- a/src/xleda/assets/xleda_template.xlsx
+++ b/src/xleda/assets/xleda_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5E2509F-FFE9-45BF-B5CD-10F078CD5CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F4C349D-DA47-4950-A680-E339A02852C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
   <sheets>
     <sheet name="SinglePlot" sheetId="30" state="hidden" r:id="rId1"/>

</xml_diff>

<commit_message>
Small API Changes Changed the vba flag from 'no_vba' to 'vba' for better semantics between the Python/CLI APIs. Default behaviors stayed the same Added 'no_vba' flag to Python API for backwards compatibility Removed 'export' command from the CLI
Website updates
Minor example updates/corrections
Moved the examples into Python or CLI tabs
Added links between configution, usage, and examples
</commit_message>
<xml_diff>
--- a/src/xleda/assets/xleda_template.xlsx
+++ b/src/xleda/assets/xleda_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F4C349D-DA47-4950-A680-E339A02852C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9087CA1B-66C6-4CB0-B2E8-501ED527FB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
   <sheets>
     <sheet name="SinglePlot" sheetId="30" state="hidden" r:id="rId1"/>

</xml_diff>

<commit_message>
Added docs link to template, version bump.
</commit_message>
<xml_diff>
--- a/src/xleda/assets/xleda_template.xlsx
+++ b/src/xleda/assets/xleda_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6F620F3-A2EF-441E-B95B-6FE651738853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{859CF5A4-6B7A-45E2-BA02-91EF99B6DD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
@@ -443,13 +443,13 @@
     <t>xleda Documentation:</t>
   </si>
   <si>
-    <t>https://github.com/InfoDesigner/xleda/</t>
-  </si>
-  <si>
     <t xml:space="preserve">► </t>
   </si>
   <si>
     <t>Overview →</t>
+  </si>
+  <si>
+    <t>https://infodesigner.github.io/xleda/</t>
   </si>
 </sst>
 </file>
@@ -1079,7 +1079,7 @@
     </xf>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" textRotation="180"/>
@@ -1405,6 +1405,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="28" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="3" fontId="32" fillId="2" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -4818,7 +4821,7 @@
     <row r="1" spans="2:16" ht="5.0999999999999996" customHeight="1"/>
     <row r="2" spans="2:16" ht="20.100000000000001" customHeight="1">
       <c r="B2" s="114" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D2" s="81"/>
     </row>
@@ -4933,7 +4936,7 @@
     </row>
     <row r="6" spans="1:28" ht="15" customHeight="1">
       <c r="B6" s="113" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C6" s="114" t="s">
         <v>93</v>
@@ -4961,10 +4964,10 @@
       <c r="K8" s="43"/>
     </row>
     <row r="9" spans="1:28" ht="30" hidden="1" customHeight="1">
-      <c r="C9" s="117" t="s">
+      <c r="C9" s="118" t="s">
         <v>104</v>
       </c>
-      <c r="D9" s="117"/>
+      <c r="D9" s="118"/>
       <c r="E9" s="43"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -4972,8 +4975,8 @@
     </row>
     <row r="10" spans="1:28" ht="15" hidden="1" customHeight="1">
       <c r="C10" s="43"/>
-      <c r="D10" s="80" t="s">
-        <v>105</v>
+      <c r="D10" s="117" t="s">
+        <v>107</v>
       </c>
       <c r="E10" s="43"/>
       <c r="F10" s="43"/>
@@ -4990,10 +4993,10 @@
     </row>
     <row r="12" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="B12" s="1"/>
-      <c r="C12" s="117" t="s">
+      <c r="C12" s="118" t="s">
         <v>95</v>
       </c>
-      <c r="D12" s="117"/>
+      <c r="D12" s="118"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
       <c r="K12" s="43"/>
@@ -5047,10 +5050,10 @@
       <c r="L19" s="38"/>
     </row>
     <row r="20" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C20" s="117" t="s">
+      <c r="C20" s="118" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="117"/>
+      <c r="D20" s="118"/>
       <c r="E20" s="78"/>
       <c r="L20" s="38"/>
     </row>
@@ -5178,10 +5181,10 @@
       <c r="Y38" s="38"/>
     </row>
     <row r="39" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C39" s="117" t="s">
+      <c r="C39" s="118" t="s">
         <v>53</v>
       </c>
-      <c r="D39" s="117"/>
+      <c r="D39" s="118"/>
       <c r="F39" s="43"/>
       <c r="G39" s="43"/>
       <c r="H39" s="43"/>
@@ -5402,7 +5405,7 @@
     <row r="55" spans="1:31" ht="15" customHeight="1" collapsed="1">
       <c r="A55" s="6"/>
       <c r="B55" s="67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>86</v>
@@ -5460,7 +5463,7 @@
     </row>
     <row r="61" spans="1:31" ht="15" customHeight="1">
       <c r="B61" s="67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>87</v>
@@ -5738,7 +5741,7 @@
     <row r="7" spans="1:8">
       <c r="A7" s="116"/>
       <c r="B7" s="82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>5</v>
@@ -5841,7 +5844,7 @@
     <row r="23" spans="1:6" outlineLevel="1">
       <c r="A23" s="116"/>
       <c r="B23" s="82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>7</v>
@@ -5930,7 +5933,7 @@
     <row r="36" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A36" s="116"/>
       <c r="B36" s="82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>16</v>
@@ -5992,7 +5995,7 @@
     <row r="46" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A46" s="116"/>
       <c r="B46" s="82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>22</v>
@@ -6085,7 +6088,7 @@
     <row r="58" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A58" s="116"/>
       <c r="B58" s="82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>27</v>
@@ -6217,7 +6220,7 @@
     <row r="69" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A69" s="116"/>
       <c r="B69" s="82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
Add basic usage to readme/version bump
</commit_message>
<xml_diff>
--- a/src/xleda/assets/xleda_template.xlsx
+++ b/src/xleda/assets/xleda_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\xleda\src\xleda\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1667CC2A-BDD0-4920-8BE1-707D24FA4ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6DFCBA43-1AEB-42AF-AF76-ECA985144494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
   <sheets>
     <sheet name="SinglePlot" sheetId="30" state="hidden" r:id="rId1"/>

</xml_diff>